<commit_message>
Correct the Engine Translation notes after IC-002
The proposal called A01 and A04 "gaps — no canonical Game Problem is reachable".
IC-002 makes that a category error in Christian's own terms: a Practice Situation
is a competitive CONTEXT in which several Game Problems emerge, not a synonym for
one, so a Learning Goal reaching nothing directly may still be well-formed
knowledge that resolves through its situations.

The measurement was right; the inference on top of it was not. Those rows now say
"the runtime cannot currently reach this", which is what was actually observed,
rather than "the knowledge is missing", which went beyond the evidence — and would
have argued a one-to-one reading he has explicitly rejected, in a workbook he is
about to review.

The mappings themselves are unchanged. Verified by regenerating both proposals
after the pass and goal-kick parser fixes and diffing: byte-identical, so no
mapping moved.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/back/data/session-planning/session-planning-model.rc1-PROPOSED-engine-translation.xlsx
+++ b/back/data/session-planning/session-planning-model.rc1-PROPOSED-engine-translation.xlsx
@@ -5600,7 +5600,7 @@
       <c r="C2" s="2" t="n"/>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>GAP — no canonical Game Problem is reachable from this goal today. The coach phrases fall to the general fallback, so the activity would be generic. Needs either vocabulary that routes it or a decision about which Game Problem it belongs to. Left blank deliberately.</t>
+          <t>UNRESOLVED — the coach phrases for this goal reach only the general fallback today, so the activity would be generic. Left blank deliberately rather than filled with a plausible ID. NOTE (revised after IC-002): this is not necessarily a missing Game Problem. IC-002 defines a Practice Situation as a competitive context in which several Game Problems emerge, so a goal at this level may resolve through its situations rather than to one problem directly. Read this row as "the runtime cannot currently reach it", not as "the knowledge is absent".</t>
         </is>
       </c>
     </row>
@@ -5650,7 +5650,7 @@
       <c r="C5" s="2" t="n"/>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>GAP — no canonical Game Problem is reachable from this goal today. The coach phrases fall to the general fallback, so the activity would be generic. Needs either vocabulary that routes it or a decision about which Game Problem it belongs to. Left blank deliberately.</t>
+          <t>UNRESOLVED — the coach phrases for this goal reach only the general fallback today, so the activity would be generic. Left blank deliberately rather than filled with a plausible ID. NOTE (revised after IC-002): this is not necessarily a missing Game Problem. IC-002 defines a Practice Situation as a competitive context in which several Game Problems emerge, so a goal at this level may resolve through its situations rather than to one problem directly. Read this row as "the runtime cannot currently reach it", not as "the knowledge is absent".</t>
         </is>
       </c>
     </row>

</xml_diff>